<commit_message>
Fixed lag on first lap. The Lag occurs on the first press of Start when opening the program. Further presses of start have no further lag
</commit_message>
<xml_diff>
--- a/Test/bin/Debug/template.xlsx
+++ b/Test/bin/Debug/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rtety\Documents\MQSpeed_Git\Live_Telemetry\Test\bin\Debug\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454A2871-BC0C-4702-8E7A-E54FFCF5E34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782E2237-BB27-4B17-85BB-24DE03A1F1E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7470" yWindow="3585" windowWidth="16200" windowHeight="9398" xr2:uid="{88753B80-B315-462C-BA62-9352797001B8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10800" windowHeight="12900" xr2:uid="{88753B80-B315-462C-BA62-9352797001B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -103,6 +103,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{19706C90-A9E3-4587-9825-3346553D4AAC}" name="Table1" displayName="Table1" ref="A1:E2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{19706C90-A9E3-4587-9825-3346553D4AAC}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{F234B5A9-2412-4589-A5A5-1129CD74C4D2}" name="Lap Number"/>
+    <tableColumn id="2" xr3:uid="{51440C30-2A92-4F23-8028-8035C4F6842B}" name="Lap Time"/>
+    <tableColumn id="3" xr3:uid="{0112C74F-59E5-49F8-98C6-588256C90487}" name="Global Start"/>
+    <tableColumn id="4" xr3:uid="{1EA015D4-6836-4441-85AB-D6ABD8133F85}" name="Global End"/>
+    <tableColumn id="5" xr3:uid="{57C1582A-52EF-4660-8D37-298B32386724}" name="Real Time"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -425,8 +439,8 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.265625" customWidth="1"/>
-    <col min="2" max="2" width="11.1328125" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.9296875" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" customWidth="1"/>
     <col min="4" max="4" width="14.46484375" customWidth="1"/>
     <col min="5" max="5" width="13.9296875" customWidth="1"/>
@@ -452,5 +466,8 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>